<commit_message>
Update AI Job Agent
</commit_message>
<xml_diff>
--- a/Jobs.xlsx
+++ b/Jobs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Add professional job scoring and clickable apply links
</commit_message>
<xml_diff>
--- a/Jobs.xlsx
+++ b/Jobs.xlsx
@@ -17,13 +17,23 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,14 +53,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,112 +427,560 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Apply</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Score</t>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Overall Score</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Telecom</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Matched Skills</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Svitzer</t>
+          <t>Sophie's Flats Inc.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chief Engineer</t>
+          <t>Architectural Designer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freeport, </t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://remoteOK.com/remote-jobs/remote-chief-engineer-svitzer-1136275</t>
+          <t xml:space="preserve">Toronto, </t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-architectural-designer-sophies-flats-inc-1136192</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>50</v>
+      </c>
+      <c r="F2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>architect, architectural, autocad, building, construction, engineer, remote, revit, sketchup</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sophie's Flats Inc.</t>
+          <t>PAXIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Architectural Designer</t>
+          <t>Page Not Found</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toronto, </t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://remoteOK.com/remote-jobs/remote-architectural-designer-sophies-flats-inc-1136192</t>
+          <t xml:space="preserve">Coral Bay, </t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-page-not-found-paxio-1136324</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>34</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>16</v>
+      </c>
+      <c r="J3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>building, customer service, customer support, internet, isp, network, telecom</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nexlane</t>
+          <t>Lemon.io</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SiteProcure</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evansville, </t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://remoteOK.com/remote-jobs/remote-siteprocure-nexlane-1136169</t>
+          <t>Senior React Full stack Developer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-senior-react-full-stack-developer-lemon-io-1136299</t>
         </is>
       </c>
       <c r="E4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>architect, engineer, engineering, remote, site</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Order From Chaos, Today!</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Donât Put Yourself a Box</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ottawa, </t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-dont-put-yourself-a-box-order-from-chaos-today-1136184</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>29</v>
+      </c>
+      <c r="F5" t="n">
+        <v>24</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>building, engineer, engineering, network</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Brand Strategy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gurgaon, </t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-brand-strategy-capgemini-1136220</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>26</v>
+      </c>
+      <c r="F6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>architect, building, network, remote</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Clera</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Java Developer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-java-developer-clera-1136188</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" t="n">
+        <v>25</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>architect, architectural, building, engineer, engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Four Seasons</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Holly Can Fix It</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nassau, </t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-holly-can-fix-it-four-seasons-1136305</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" t="n">
+        <v>24</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>building, engineer, engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>The Well</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Joel Q</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edmonton, </t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-joel-q-the-well-1136288</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" t="n">
+        <v>24</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>building, engineer, engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Simmons Civil</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Labourers</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gladstone, </t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-labourers-simmons-civil-1136230</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>24</v>
+      </c>
+      <c r="F10" t="n">
+        <v>24</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>civil, construction, site</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tridant</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>owlette</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fleet, </t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-owlette-tridant-1136206</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>23</v>
+      </c>
+      <c r="F11" t="n">
         <v>8</v>
       </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>internet, isp, network, remote, site</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add jobicy integration and multi-source job search
</commit_message>
<xml_diff>
--- a/Jobs.xlsx
+++ b/Jobs.xlsx
@@ -495,124 +495,128 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sophie's Flats Inc.</t>
+          <t>Elevenlabs</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Architectural Designer</t>
+          <t>Account Executive - Canada - Enterprise</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toronto, </t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-architectural-designer-sophies-flats-inc-1136192</t>
+          <t>https://jobicy.com/jobs/148827-account-executive-canada-enterprise</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F2" t="n">
         <v>25</v>
       </c>
       <c r="G2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K2" t="n">
         <v>5</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>architect, architectural, autocad, building, construction, engineer, remote, revit, sketchup</t>
+          <t>building, customer support, engineer, engineering, remote, sales, site, telecom</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PAXIO</t>
+          <t>Planet Labs Inc.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Page Not Found</t>
+          <t>Senior Solutions Architect I, Pre-Sales - South Korea Defense &amp; Intelligence</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coral Bay, </t>
+          <t>APAC</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-page-not-found-paxio-1136324</t>
+          <t>https://jobicy.com/jobs/148688-senior-solutions-architect-i-pre-sales-south-korea-defense-intelligence</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>building, customer service, customer support, internet, isp, network, telecom</t>
+          <t>architect, building, business development, engineer, engineering, internet, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
+          <t>Sophie's Flats Inc.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Senior React Full stack Developer</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Architectural Designer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Toronto, </t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-senior-react-full-stack-developer-lemon-io-1136299</t>
+          <t>https://remoteOK.com/remote-jobs/remote-architectural-designer-sophies-flats-inc-1136192</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F4" t="n">
         <v>25</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -628,225 +632,225 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>architect, engineer, engineering, remote, site</t>
+          <t>architect, architectural, autocad, building, construction, engineer, remote, revit, sketchup</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Order From Chaos, Today!</t>
+          <t>Samsara</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Donât Put Yourself a Box</t>
+          <t>Enterprise Sales Engineer - Toronto</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ottawa, </t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-dont-put-yourself-a-box-order-from-chaos-today-1136184</t>
+          <t>https://jobicy.com/jobs/142074-enterprise-sales-engineer-toronto</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="F5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>building, engineer, engineering, network</t>
+          <t>building, construction, engineer, engineering, internet, network, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Zscaler</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Brand Strategy</t>
+          <t>Transformation Architect - Healthcare</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gurgaon, </t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-brand-strategy-capgemini-1136220</t>
+          <t>https://jobicy.com/jobs/145317-transformation-architect-healthcare</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="F6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K6" t="n">
         <v>5</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>architect, building, network, remote</t>
+          <t>architect, building, isp, network, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Clera</t>
+          <t>CrowdStrike</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Java Developer</t>
+          <t>Technical Account Manager II - Customer Onboarding</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-java-developer-clera-1136188</t>
+          <t>https://jobicy.com/jobs/148743-technical-account-manager-ii-customer-onboarding</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>architect, architectural, building, engineer, engineering</t>
+          <t>customer service, engineer, internet, network, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Four Seasons</t>
+          <t>Elevenlabs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Holly Can Fix It</t>
+          <t>Account Executive - Canada - Corporate</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nassau, </t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-holly-can-fix-it-four-seasons-1136305</t>
+          <t>https://jobicy.com/jobs/148829-account-executive-canada-corporate</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>building, engineer, engineering</t>
+          <t>building, customer support, engineer, engineering, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The Well</t>
+          <t>Sumsub</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joel Q</t>
+          <t>Junior Customer Success Manager</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edmonton, </t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-joel-q-the-well-1136288</t>
+          <t>https://jobicy.com/jobs/150276-junior-customer-success-manager</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="F9" t="n">
         <v>24</v>
@@ -855,7 +859,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -864,107 +868,107 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>building, engineer, engineering</t>
+          <t>architect, building, business development, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Simmons Civil</t>
+          <t>Samsara</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Labourers</t>
+          <t>Customer Success Manager III</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gladstone, </t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-labourers-simmons-civil-1136230</t>
+          <t>https://jobicy.com/jobs/148927-customer-success-manager-iii</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="F10" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>civil, construction, site</t>
+          <t>architect, building, construction, engineer, engineering, internet, remote, sales, site</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tridant</t>
+          <t>Voyage Privé</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>owlette</t>
+          <t>Security Engineer - Full Remote (France) or Hybrid</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fleet, </t>
+          <t>France</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-owlette-tridant-1136206</t>
+          <t>https://jobicy.com/jobs/145653-security-engineer-full-remote-france-or-hybrid</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="F11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>8</v>
       </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K11" t="n">
         <v>5</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>internet, isp, network, remote, site</t>
+          <t>architect, architectural, business development, engineer, engineering, network, remote, site</t>
         </is>
       </c>
     </row>

</xml_diff>